<commit_message>
Updated POL_grids_kan50 model - 2026-10-03 19:45
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/Sets-vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA0DA4AE-49E8-4516-A18B-DB30EE822310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F49DC8-A038-4969-AF13-4EE05F54EB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="943" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="557">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -538,12 +538,6 @@
     <t>*[_]Legnica_POL</t>
   </si>
   <si>
-    <t>p_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>*[_]Olesnica_POL</t>
-  </si>
-  <si>
     <t>p_Swidnica_POL</t>
   </si>
   <si>
@@ -610,12 +604,6 @@
     <t>*[_]Grajewo_POL</t>
   </si>
   <si>
-    <t>p_PiotrkowTrybunalsk_POL</t>
-  </si>
-  <si>
-    <t>*[_]PiotrkowTrybunalsk_POL</t>
-  </si>
-  <si>
     <t>p_Radomsko_POL</t>
   </si>
   <si>
@@ -658,12 +646,6 @@
     <t>*[_]Chelm_POL</t>
   </si>
   <si>
-    <t>p_Debica_POL</t>
-  </si>
-  <si>
-    <t>*[_]Debica_POL</t>
-  </si>
-  <si>
     <t>p_Kielce_POL</t>
   </si>
   <si>
@@ -724,12 +706,6 @@
     <t>*[_]Warsaw_POL</t>
   </si>
   <si>
-    <t>p_Gliwice_POL</t>
-  </si>
-  <si>
-    <t>*[_]Gliwice_POL</t>
-  </si>
-  <si>
     <t>p_Elk_POL</t>
   </si>
   <si>
@@ -1282,6 +1258,66 @@
     <t>elc_wof_POL_010</t>
   </si>
   <si>
+    <t>p_Siedlce_POL</t>
+  </si>
+  <si>
+    <t>*[_]Siedlce_POL</t>
+  </si>
+  <si>
+    <t>p_Lukow_POL</t>
+  </si>
+  <si>
+    <t>*[_]Lukow_POL</t>
+  </si>
+  <si>
+    <t>p_Ostroleka_POL</t>
+  </si>
+  <si>
+    <t>*[_]Ostroleka_POL</t>
+  </si>
+  <si>
+    <t>p_Lublin_POL</t>
+  </si>
+  <si>
+    <t>*[_]Lublin_POL</t>
+  </si>
+  <si>
+    <t>p_Radom_POL</t>
+  </si>
+  <si>
+    <t>*[_]Radom_POL</t>
+  </si>
+  <si>
+    <t>p_Pila_POL</t>
+  </si>
+  <si>
+    <t>*[_]Pila_POL</t>
+  </si>
+  <si>
+    <t>p_Kalisz_POL</t>
+  </si>
+  <si>
+    <t>*[_]Kalisz_POL</t>
+  </si>
+  <si>
+    <t>p_Walbrzych_POL</t>
+  </si>
+  <si>
+    <t>*[_]Walbrzych_POL</t>
+  </si>
+  <si>
+    <t>p_Belchatow_POL</t>
+  </si>
+  <si>
+    <t>*[_]Belchatow_POL</t>
+  </si>
+  <si>
+    <t>p_Lodz_POL</t>
+  </si>
+  <si>
+    <t>*[_]Lodz_POL</t>
+  </si>
+  <si>
     <t>rez_spv_POL_021</t>
   </si>
   <si>
@@ -1450,6 +1486,36 @@
     <t>elc_spv_POL_048</t>
   </si>
   <si>
+    <t>rez_spv_POL_049</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_049</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_050</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_050</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_051</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_051</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_052</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_052</t>
+  </si>
+  <si>
+    <t>rez_spv_POL_053</t>
+  </si>
+  <si>
+    <t>elc_spv_POL_053</t>
+  </si>
+  <si>
     <t>rez_won_POL_021</t>
   </si>
   <si>
@@ -1616,6 +1682,30 @@
   </si>
   <si>
     <t>elc_won_POL_048</t>
+  </si>
+  <si>
+    <t>rez_won_POL_049</t>
+  </si>
+  <si>
+    <t>elc_won_POL_049</t>
+  </si>
+  <si>
+    <t>rez_won_POL_050</t>
+  </si>
+  <si>
+    <t>elc_won_POL_050</t>
+  </si>
+  <si>
+    <t>rez_won_POL_051</t>
+  </si>
+  <si>
+    <t>elc_won_POL_051</t>
+  </si>
+  <si>
+    <t>rez_won_POL_052</t>
+  </si>
+  <si>
+    <t>elc_won_POL_052</t>
   </si>
 </sst>
 </file>
@@ -2191,7 +2281,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B9:E194"/>
+  <dimension ref="B9:E209"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -2257,13 +2347,13 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>165</v>
+        <v>407</v>
       </c>
       <c r="C14" t="s">
-        <v>166</v>
+        <v>408</v>
       </c>
       <c r="D14" t="s">
-        <v>166</v>
+        <v>408</v>
       </c>
       <c r="E14" t="s">
         <v>160</v>
@@ -2271,13 +2361,13 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>167</v>
+        <v>409</v>
       </c>
       <c r="C15" t="s">
-        <v>168</v>
+        <v>410</v>
       </c>
       <c r="D15" t="s">
-        <v>168</v>
+        <v>410</v>
       </c>
       <c r="E15" t="s">
         <v>160</v>
@@ -2285,13 +2375,13 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E16" t="s">
         <v>160</v>
@@ -2299,13 +2389,13 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C17" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E17" t="s">
         <v>160</v>
@@ -2313,13 +2403,13 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="C18" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D18" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="E18" t="s">
         <v>160</v>
@@ -2327,13 +2417,13 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C19" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D19" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E19" t="s">
         <v>160</v>
@@ -2341,13 +2431,13 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C20" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D20" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E20" t="s">
         <v>160</v>
@@ -2355,13 +2445,13 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C21" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D21" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="E21" t="s">
         <v>160</v>
@@ -2369,13 +2459,13 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C22" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D22" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="E22" t="s">
         <v>160</v>
@@ -2383,13 +2473,13 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E23" t="s">
         <v>160</v>
@@ -2397,13 +2487,13 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>185</v>
+        <v>411</v>
       </c>
       <c r="C24" t="s">
-        <v>186</v>
+        <v>412</v>
       </c>
       <c r="D24" t="s">
-        <v>186</v>
+        <v>412</v>
       </c>
       <c r="E24" t="s">
         <v>160</v>
@@ -2411,13 +2501,13 @@
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C25" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D25" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E25" t="s">
         <v>160</v>
@@ -2425,13 +2515,13 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C26" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D26" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="E26" t="s">
         <v>160</v>
@@ -2439,13 +2529,13 @@
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C27" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D27" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="E27" t="s">
         <v>160</v>
@@ -2453,13 +2543,13 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>193</v>
+        <v>413</v>
       </c>
       <c r="C28" t="s">
-        <v>194</v>
+        <v>414</v>
       </c>
       <c r="D28" t="s">
-        <v>194</v>
+        <v>414</v>
       </c>
       <c r="E28" t="s">
         <v>160</v>
@@ -2467,13 +2557,13 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C29" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D29" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="E29" t="s">
         <v>160</v>
@@ -2481,13 +2571,13 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C30" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D30" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E30" t="s">
         <v>160</v>
@@ -2495,13 +2585,13 @@
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="C31" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D31" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="E31" t="s">
         <v>160</v>
@@ -2509,13 +2599,13 @@
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>201</v>
+        <v>415</v>
       </c>
       <c r="C32" t="s">
-        <v>202</v>
+        <v>416</v>
       </c>
       <c r="D32" t="s">
-        <v>202</v>
+        <v>416</v>
       </c>
       <c r="E32" t="s">
         <v>160</v>
@@ -2523,13 +2613,13 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="C33" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="D33" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="E33" t="s">
         <v>160</v>
@@ -2537,13 +2627,13 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C34" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="D34" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="E34" t="s">
         <v>160</v>
@@ -2551,13 +2641,13 @@
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B35" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="C35" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="D35" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="E35" t="s">
         <v>160</v>
@@ -2565,13 +2655,13 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B36" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C36" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D36" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E36" t="s">
         <v>160</v>
@@ -2579,13 +2669,13 @@
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B37" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C37" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D37" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E37" t="s">
         <v>160</v>
@@ -2593,13 +2683,13 @@
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B38" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C38" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D38" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="E38" t="s">
         <v>160</v>
@@ -2607,13 +2697,13 @@
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B39" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C39" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="D39" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="E39" t="s">
         <v>160</v>
@@ -2621,13 +2711,13 @@
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B40" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="C40" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D40" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="E40" t="s">
         <v>160</v>
@@ -2635,13 +2725,13 @@
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="C41" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D41" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="E41" t="s">
         <v>160</v>
@@ -2649,13 +2739,13 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" t="s">
-        <v>221</v>
+        <v>417</v>
       </c>
       <c r="C42" t="s">
-        <v>222</v>
+        <v>418</v>
       </c>
       <c r="D42" t="s">
-        <v>222</v>
+        <v>418</v>
       </c>
       <c r="E42" t="s">
         <v>160</v>
@@ -2663,13 +2753,13 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C43" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="D43" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="E43" t="s">
         <v>160</v>
@@ -2677,13 +2767,13 @@
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="C44" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="D44" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="E44" t="s">
         <v>160</v>
@@ -2691,13 +2781,13 @@
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="C45" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="D45" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="E45" t="s">
         <v>160</v>
@@ -2705,13 +2795,13 @@
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C46" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="D46" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="E46" t="s">
         <v>160</v>
@@ -2719,13 +2809,13 @@
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" t="s">
-        <v>231</v>
+        <v>419</v>
       </c>
       <c r="C47" t="s">
-        <v>232</v>
+        <v>420</v>
       </c>
       <c r="D47" t="s">
-        <v>232</v>
+        <v>420</v>
       </c>
       <c r="E47" t="s">
         <v>160</v>
@@ -2733,13 +2823,13 @@
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="C48" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="D48" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="E48" t="s">
         <v>160</v>
@@ -2747,13 +2837,13 @@
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" t="s">
-        <v>235</v>
+        <v>421</v>
       </c>
       <c r="C49" t="s">
-        <v>236</v>
+        <v>422</v>
       </c>
       <c r="D49" t="s">
-        <v>236</v>
+        <v>422</v>
       </c>
       <c r="E49" t="s">
         <v>160</v>
@@ -2761,13 +2851,13 @@
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="C50" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="D50" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="E50" t="s">
         <v>160</v>
@@ -2775,13 +2865,13 @@
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" t="s">
-        <v>239</v>
+        <v>423</v>
       </c>
       <c r="C51" t="s">
-        <v>240</v>
+        <v>424</v>
       </c>
       <c r="D51" t="s">
-        <v>240</v>
+        <v>424</v>
       </c>
       <c r="E51" t="s">
         <v>160</v>
@@ -2789,13 +2879,13 @@
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B52" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="C52" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="D52" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="E52" t="s">
         <v>160</v>
@@ -2803,13 +2893,13 @@
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B53" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="C53" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="D53" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="E53" t="s">
         <v>160</v>
@@ -2817,13 +2907,13 @@
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B54" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="C54" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="D54" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="E54" t="s">
         <v>160</v>
@@ -2831,13 +2921,13 @@
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B55" t="s">
-        <v>247</v>
+        <v>425</v>
       </c>
       <c r="C55" t="s">
-        <v>248</v>
+        <v>426</v>
       </c>
       <c r="D55" t="s">
-        <v>248</v>
+        <v>426</v>
       </c>
       <c r="E55" t="s">
         <v>160</v>
@@ -2845,13 +2935,13 @@
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B56" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="C56" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="D56" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="E56" t="s">
         <v>160</v>
@@ -2859,13 +2949,13 @@
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B57" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="C57" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="D57" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="E57" t="s">
         <v>160</v>
@@ -2873,13 +2963,13 @@
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B58" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="C58" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="D58" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="E58" t="s">
         <v>160</v>
@@ -2887,13 +2977,13 @@
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B59" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="C59" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="D59" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="E59" t="s">
         <v>160</v>
@@ -2901,13 +2991,13 @@
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B60" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="C60" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="D60" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="E60" t="s">
         <v>160</v>
@@ -2915,13 +3005,13 @@
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B61" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="C61" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="D61" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="E61" t="s">
         <v>160</v>
@@ -2929,13 +3019,13 @@
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B62" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="C62" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="D62" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="E62" t="s">
         <v>160</v>
@@ -2943,13 +3033,13 @@
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B63" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C63" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="D63" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="E63" t="s">
         <v>160</v>
@@ -2957,13 +3047,13 @@
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B64" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="C64" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="D64" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="E64" t="s">
         <v>160</v>
@@ -2971,13 +3061,13 @@
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B65" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="C65" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="D65" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="E65" t="s">
         <v>160</v>
@@ -2985,13 +3075,13 @@
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B66" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="C66" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="D66" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="E66" t="s">
         <v>160</v>
@@ -2999,13 +3089,13 @@
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B67" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="C67" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="D67" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="E67" t="s">
         <v>160</v>
@@ -3013,13 +3103,13 @@
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B68" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="C68" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="D68" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="E68" t="s">
         <v>160</v>
@@ -3027,13 +3117,13 @@
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B69" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="C69" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="D69" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="E69" t="s">
         <v>160</v>
@@ -3041,13 +3131,13 @@
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B70" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="C70" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="D70" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="E70" t="s">
         <v>160</v>
@@ -3055,13 +3145,13 @@
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B71" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
       <c r="C71" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="D71" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="E71" t="s">
         <v>160</v>
@@ -3069,13 +3159,13 @@
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B72" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="C72" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="D72" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="E72" t="s">
         <v>160</v>
@@ -3083,13 +3173,13 @@
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B73" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="C73" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="D73" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="E73" t="s">
         <v>160</v>
@@ -3097,13 +3187,13 @@
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B74" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
       <c r="C74" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
       <c r="D74" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
       <c r="E74" t="s">
         <v>160</v>
@@ -3111,13 +3201,13 @@
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B75" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
       <c r="C75" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="D75" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="E75" t="s">
         <v>160</v>
@@ -3125,13 +3215,13 @@
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B76" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="C76" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="D76" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="E76" t="s">
         <v>160</v>
@@ -3139,13 +3229,13 @@
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B77" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
       <c r="C77" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
       <c r="D77" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
       <c r="E77" t="s">
         <v>160</v>
@@ -3153,13 +3243,13 @@
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B78" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
       <c r="C78" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="D78" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="E78" t="s">
         <v>160</v>
@@ -3167,13 +3257,13 @@
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B79" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="C79" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="D79" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="E79" t="s">
         <v>160</v>
@@ -3181,13 +3271,13 @@
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B80" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="C80" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="D80" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="E80" t="s">
         <v>160</v>
@@ -3195,13 +3285,13 @@
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B81" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="C81" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="D81" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="E81" t="s">
         <v>160</v>
@@ -3209,13 +3299,13 @@
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B82" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="C82" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="D82" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="E82" t="s">
         <v>160</v>
@@ -3223,13 +3313,13 @@
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B83" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="C83" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="D83" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="E83" t="s">
         <v>160</v>
@@ -3237,13 +3327,13 @@
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B84" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="C84" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
       <c r="D84" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
       <c r="E84" t="s">
         <v>160</v>
@@ -3251,13 +3341,13 @@
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B85" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="C85" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="D85" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="E85" t="s">
         <v>160</v>
@@ -3265,13 +3355,13 @@
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B86" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="C86" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="D86" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="E86" t="s">
         <v>160</v>
@@ -3279,13 +3369,13 @@
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B87" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
       <c r="C87" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="D87" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="E87" t="s">
         <v>160</v>
@@ -3293,13 +3383,13 @@
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B88" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="C88" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="D88" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="E88" t="s">
         <v>160</v>
@@ -3307,13 +3397,13 @@
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B89" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="C89" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="D89" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="E89" t="s">
         <v>160</v>
@@ -3321,13 +3411,13 @@
     </row>
     <row r="90" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B90" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="C90" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="D90" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="E90" t="s">
         <v>160</v>
@@ -3335,13 +3425,13 @@
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B91" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="C91" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="D91" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="E91" t="s">
         <v>160</v>
@@ -3349,13 +3439,13 @@
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B92" t="s">
-        <v>321</v>
+        <v>301</v>
       </c>
       <c r="C92" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
       <c r="D92" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
       <c r="E92" t="s">
         <v>160</v>
@@ -3363,13 +3453,13 @@
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B93" t="s">
-        <v>323</v>
+        <v>303</v>
       </c>
       <c r="C93" t="s">
-        <v>324</v>
+        <v>304</v>
       </c>
       <c r="D93" t="s">
-        <v>324</v>
+        <v>304</v>
       </c>
       <c r="E93" t="s">
         <v>160</v>
@@ -3377,13 +3467,13 @@
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B94" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C94" t="s">
-        <v>326</v>
+        <v>306</v>
       </c>
       <c r="D94" t="s">
-        <v>326</v>
+        <v>306</v>
       </c>
       <c r="E94" t="s">
         <v>160</v>
@@ -3391,13 +3481,13 @@
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B95" t="s">
-        <v>327</v>
+        <v>307</v>
       </c>
       <c r="C95" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
       <c r="D95" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
       <c r="E95" t="s">
         <v>160</v>
@@ -3405,13 +3495,13 @@
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B96" t="s">
-        <v>329</v>
+        <v>309</v>
       </c>
       <c r="C96" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
       <c r="D96" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
       <c r="E96" t="s">
         <v>160</v>
@@ -3419,13 +3509,13 @@
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B97" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="C97" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
       <c r="D97" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
       <c r="E97" t="s">
         <v>160</v>
@@ -3433,13 +3523,13 @@
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B98" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C98" t="s">
-        <v>334</v>
+        <v>314</v>
       </c>
       <c r="D98" t="s">
-        <v>334</v>
+        <v>314</v>
       </c>
       <c r="E98" t="s">
         <v>160</v>
@@ -3447,13 +3537,13 @@
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B99" t="s">
-        <v>335</v>
+        <v>315</v>
       </c>
       <c r="C99" t="s">
-        <v>336</v>
+        <v>316</v>
       </c>
       <c r="D99" t="s">
-        <v>336</v>
+        <v>316</v>
       </c>
       <c r="E99" t="s">
         <v>160</v>
@@ -3461,13 +3551,13 @@
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B100" t="s">
-        <v>337</v>
+        <v>317</v>
       </c>
       <c r="C100" t="s">
-        <v>338</v>
+        <v>318</v>
       </c>
       <c r="D100" t="s">
-        <v>338</v>
+        <v>318</v>
       </c>
       <c r="E100" t="s">
         <v>160</v>
@@ -3475,13 +3565,13 @@
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B101" t="s">
-        <v>339</v>
+        <v>319</v>
       </c>
       <c r="C101" t="s">
-        <v>340</v>
+        <v>320</v>
       </c>
       <c r="D101" t="s">
-        <v>340</v>
+        <v>320</v>
       </c>
       <c r="E101" t="s">
         <v>160</v>
@@ -3489,13 +3579,13 @@
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B102" t="s">
-        <v>341</v>
+        <v>321</v>
       </c>
       <c r="C102" t="s">
-        <v>342</v>
+        <v>322</v>
       </c>
       <c r="D102" t="s">
-        <v>342</v>
+        <v>322</v>
       </c>
       <c r="E102" t="s">
         <v>160</v>
@@ -3503,13 +3593,13 @@
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B103" t="s">
-        <v>343</v>
+        <v>323</v>
       </c>
       <c r="C103" t="s">
-        <v>344</v>
+        <v>324</v>
       </c>
       <c r="D103" t="s">
-        <v>344</v>
+        <v>324</v>
       </c>
       <c r="E103" t="s">
         <v>160</v>
@@ -3517,13 +3607,13 @@
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B104" t="s">
-        <v>345</v>
+        <v>325</v>
       </c>
       <c r="C104" t="s">
-        <v>346</v>
+        <v>326</v>
       </c>
       <c r="D104" t="s">
-        <v>346</v>
+        <v>326</v>
       </c>
       <c r="E104" t="s">
         <v>160</v>
@@ -3531,13 +3621,13 @@
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B105" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
       <c r="C105" t="s">
-        <v>348</v>
+        <v>328</v>
       </c>
       <c r="D105" t="s">
-        <v>348</v>
+        <v>328</v>
       </c>
       <c r="E105" t="s">
         <v>160</v>
@@ -3545,13 +3635,13 @@
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B106" t="s">
-        <v>349</v>
+        <v>329</v>
       </c>
       <c r="C106" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="D106" t="s">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="E106" t="s">
         <v>160</v>
@@ -3559,13 +3649,13 @@
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B107" t="s">
-        <v>351</v>
+        <v>331</v>
       </c>
       <c r="C107" t="s">
-        <v>352</v>
+        <v>332</v>
       </c>
       <c r="D107" t="s">
-        <v>352</v>
+        <v>332</v>
       </c>
       <c r="E107" t="s">
         <v>160</v>
@@ -3573,13 +3663,13 @@
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B108" t="s">
-        <v>353</v>
+        <v>333</v>
       </c>
       <c r="C108" t="s">
-        <v>354</v>
+        <v>334</v>
       </c>
       <c r="D108" t="s">
-        <v>354</v>
+        <v>334</v>
       </c>
       <c r="E108" t="s">
         <v>160</v>
@@ -3587,13 +3677,13 @@
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B109" t="s">
-        <v>415</v>
+        <v>335</v>
       </c>
       <c r="C109" t="s">
-        <v>416</v>
+        <v>336</v>
       </c>
       <c r="D109" t="s">
-        <v>416</v>
+        <v>336</v>
       </c>
       <c r="E109" t="s">
         <v>160</v>
@@ -3601,13 +3691,13 @@
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B110" t="s">
-        <v>417</v>
+        <v>337</v>
       </c>
       <c r="C110" t="s">
-        <v>418</v>
+        <v>338</v>
       </c>
       <c r="D110" t="s">
-        <v>418</v>
+        <v>338</v>
       </c>
       <c r="E110" t="s">
         <v>160</v>
@@ -3615,13 +3705,13 @@
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B111" t="s">
-        <v>419</v>
+        <v>339</v>
       </c>
       <c r="C111" t="s">
-        <v>420</v>
+        <v>340</v>
       </c>
       <c r="D111" t="s">
-        <v>420</v>
+        <v>340</v>
       </c>
       <c r="E111" t="s">
         <v>160</v>
@@ -3629,13 +3719,13 @@
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B112" t="s">
-        <v>421</v>
+        <v>341</v>
       </c>
       <c r="C112" t="s">
-        <v>422</v>
+        <v>342</v>
       </c>
       <c r="D112" t="s">
-        <v>422</v>
+        <v>342</v>
       </c>
       <c r="E112" t="s">
         <v>160</v>
@@ -3643,13 +3733,13 @@
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B113" t="s">
-        <v>423</v>
+        <v>343</v>
       </c>
       <c r="C113" t="s">
-        <v>424</v>
+        <v>344</v>
       </c>
       <c r="D113" t="s">
-        <v>424</v>
+        <v>344</v>
       </c>
       <c r="E113" t="s">
         <v>160</v>
@@ -3657,13 +3747,13 @@
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B114" t="s">
-        <v>425</v>
+        <v>345</v>
       </c>
       <c r="C114" t="s">
-        <v>426</v>
+        <v>346</v>
       </c>
       <c r="D114" t="s">
-        <v>426</v>
+        <v>346</v>
       </c>
       <c r="E114" t="s">
         <v>160</v>
@@ -3979,13 +4069,13 @@
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B137" t="s">
-        <v>355</v>
+        <v>471</v>
       </c>
       <c r="C137" t="s">
-        <v>356</v>
+        <v>472</v>
       </c>
       <c r="D137" t="s">
-        <v>356</v>
+        <v>472</v>
       </c>
       <c r="E137" t="s">
         <v>160</v>
@@ -3993,13 +4083,13 @@
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B138" t="s">
-        <v>357</v>
+        <v>473</v>
       </c>
       <c r="C138" t="s">
-        <v>358</v>
+        <v>474</v>
       </c>
       <c r="D138" t="s">
-        <v>358</v>
+        <v>474</v>
       </c>
       <c r="E138" t="s">
         <v>160</v>
@@ -4007,13 +4097,13 @@
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B139" t="s">
-        <v>359</v>
+        <v>475</v>
       </c>
       <c r="C139" t="s">
-        <v>360</v>
+        <v>476</v>
       </c>
       <c r="D139" t="s">
-        <v>360</v>
+        <v>476</v>
       </c>
       <c r="E139" t="s">
         <v>160</v>
@@ -4021,13 +4111,13 @@
     </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B140" t="s">
-        <v>361</v>
+        <v>477</v>
       </c>
       <c r="C140" t="s">
-        <v>362</v>
+        <v>478</v>
       </c>
       <c r="D140" t="s">
-        <v>362</v>
+        <v>478</v>
       </c>
       <c r="E140" t="s">
         <v>160</v>
@@ -4035,13 +4125,13 @@
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B141" t="s">
-        <v>363</v>
+        <v>479</v>
       </c>
       <c r="C141" t="s">
-        <v>364</v>
+        <v>480</v>
       </c>
       <c r="D141" t="s">
-        <v>364</v>
+        <v>480</v>
       </c>
       <c r="E141" t="s">
         <v>160</v>
@@ -4049,13 +4139,13 @@
     </row>
     <row r="142" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B142" t="s">
-        <v>365</v>
+        <v>481</v>
       </c>
       <c r="C142" t="s">
-        <v>366</v>
+        <v>482</v>
       </c>
       <c r="D142" t="s">
-        <v>366</v>
+        <v>482</v>
       </c>
       <c r="E142" t="s">
         <v>160</v>
@@ -4063,13 +4153,13 @@
     </row>
     <row r="143" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B143" t="s">
-        <v>367</v>
+        <v>483</v>
       </c>
       <c r="C143" t="s">
-        <v>368</v>
+        <v>484</v>
       </c>
       <c r="D143" t="s">
-        <v>368</v>
+        <v>484</v>
       </c>
       <c r="E143" t="s">
         <v>160</v>
@@ -4077,13 +4167,13 @@
     </row>
     <row r="144" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B144" t="s">
-        <v>369</v>
+        <v>485</v>
       </c>
       <c r="C144" t="s">
-        <v>370</v>
+        <v>486</v>
       </c>
       <c r="D144" t="s">
-        <v>370</v>
+        <v>486</v>
       </c>
       <c r="E144" t="s">
         <v>160</v>
@@ -4091,13 +4181,13 @@
     </row>
     <row r="145" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B145" t="s">
-        <v>371</v>
+        <v>487</v>
       </c>
       <c r="C145" t="s">
-        <v>372</v>
+        <v>488</v>
       </c>
       <c r="D145" t="s">
-        <v>372</v>
+        <v>488</v>
       </c>
       <c r="E145" t="s">
         <v>160</v>
@@ -4105,13 +4195,13 @@
     </row>
     <row r="146" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B146" t="s">
-        <v>373</v>
+        <v>489</v>
       </c>
       <c r="C146" t="s">
-        <v>374</v>
+        <v>490</v>
       </c>
       <c r="D146" t="s">
-        <v>374</v>
+        <v>490</v>
       </c>
       <c r="E146" t="s">
         <v>160</v>
@@ -4119,13 +4209,13 @@
     </row>
     <row r="147" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B147" t="s">
-        <v>375</v>
+        <v>491</v>
       </c>
       <c r="C147" t="s">
-        <v>376</v>
+        <v>492</v>
       </c>
       <c r="D147" t="s">
-        <v>376</v>
+        <v>492</v>
       </c>
       <c r="E147" t="s">
         <v>160</v>
@@ -4133,13 +4223,13 @@
     </row>
     <row r="148" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B148" t="s">
-        <v>377</v>
+        <v>347</v>
       </c>
       <c r="C148" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="D148" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="E148" t="s">
         <v>160</v>
@@ -4147,13 +4237,13 @@
     </row>
     <row r="149" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B149" t="s">
-        <v>379</v>
+        <v>349</v>
       </c>
       <c r="C149" t="s">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="D149" t="s">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="E149" t="s">
         <v>160</v>
@@ -4161,13 +4251,13 @@
     </row>
     <row r="150" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B150" t="s">
-        <v>381</v>
+        <v>351</v>
       </c>
       <c r="C150" t="s">
-        <v>382</v>
+        <v>352</v>
       </c>
       <c r="D150" t="s">
-        <v>382</v>
+        <v>352</v>
       </c>
       <c r="E150" t="s">
         <v>160</v>
@@ -4175,13 +4265,13 @@
     </row>
     <row r="151" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B151" t="s">
-        <v>383</v>
+        <v>353</v>
       </c>
       <c r="C151" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="D151" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="E151" t="s">
         <v>160</v>
@@ -4189,13 +4279,13 @@
     </row>
     <row r="152" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B152" t="s">
-        <v>385</v>
+        <v>355</v>
       </c>
       <c r="C152" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="D152" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="E152" t="s">
         <v>160</v>
@@ -4203,13 +4293,13 @@
     </row>
     <row r="153" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B153" t="s">
-        <v>387</v>
+        <v>357</v>
       </c>
       <c r="C153" t="s">
-        <v>388</v>
+        <v>358</v>
       </c>
       <c r="D153" t="s">
-        <v>388</v>
+        <v>358</v>
       </c>
       <c r="E153" t="s">
         <v>160</v>
@@ -4217,13 +4307,13 @@
     </row>
     <row r="154" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B154" t="s">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="C154" t="s">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="D154" t="s">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="E154" t="s">
         <v>160</v>
@@ -4231,13 +4321,13 @@
     </row>
     <row r="155" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B155" t="s">
-        <v>391</v>
+        <v>361</v>
       </c>
       <c r="C155" t="s">
-        <v>392</v>
+        <v>362</v>
       </c>
       <c r="D155" t="s">
-        <v>392</v>
+        <v>362</v>
       </c>
       <c r="E155" t="s">
         <v>160</v>
@@ -4245,13 +4335,13 @@
     </row>
     <row r="156" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B156" t="s">
-        <v>393</v>
+        <v>363</v>
       </c>
       <c r="C156" t="s">
-        <v>394</v>
+        <v>364</v>
       </c>
       <c r="D156" t="s">
-        <v>394</v>
+        <v>364</v>
       </c>
       <c r="E156" t="s">
         <v>160</v>
@@ -4259,13 +4349,13 @@
     </row>
     <row r="157" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B157" t="s">
-        <v>471</v>
+        <v>365</v>
       </c>
       <c r="C157" t="s">
-        <v>472</v>
+        <v>366</v>
       </c>
       <c r="D157" t="s">
-        <v>472</v>
+        <v>366</v>
       </c>
       <c r="E157" t="s">
         <v>160</v>
@@ -4273,13 +4363,13 @@
     </row>
     <row r="158" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B158" t="s">
-        <v>473</v>
+        <v>367</v>
       </c>
       <c r="C158" t="s">
-        <v>474</v>
+        <v>368</v>
       </c>
       <c r="D158" t="s">
-        <v>474</v>
+        <v>368</v>
       </c>
       <c r="E158" t="s">
         <v>160</v>
@@ -4287,13 +4377,13 @@
     </row>
     <row r="159" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B159" t="s">
-        <v>475</v>
+        <v>369</v>
       </c>
       <c r="C159" t="s">
-        <v>476</v>
+        <v>370</v>
       </c>
       <c r="D159" t="s">
-        <v>476</v>
+        <v>370</v>
       </c>
       <c r="E159" t="s">
         <v>160</v>
@@ -4301,13 +4391,13 @@
     </row>
     <row r="160" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B160" t="s">
-        <v>477</v>
+        <v>371</v>
       </c>
       <c r="C160" t="s">
-        <v>478</v>
+        <v>372</v>
       </c>
       <c r="D160" t="s">
-        <v>478</v>
+        <v>372</v>
       </c>
       <c r="E160" t="s">
         <v>160</v>
@@ -4315,13 +4405,13 @@
     </row>
     <row r="161" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B161" t="s">
-        <v>479</v>
+        <v>373</v>
       </c>
       <c r="C161" t="s">
-        <v>480</v>
+        <v>374</v>
       </c>
       <c r="D161" t="s">
-        <v>480</v>
+        <v>374</v>
       </c>
       <c r="E161" t="s">
         <v>160</v>
@@ -4329,13 +4419,13 @@
     </row>
     <row r="162" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B162" t="s">
-        <v>481</v>
+        <v>375</v>
       </c>
       <c r="C162" t="s">
-        <v>482</v>
+        <v>376</v>
       </c>
       <c r="D162" t="s">
-        <v>482</v>
+        <v>376</v>
       </c>
       <c r="E162" t="s">
         <v>160</v>
@@ -4343,13 +4433,13 @@
     </row>
     <row r="163" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B163" t="s">
-        <v>483</v>
+        <v>377</v>
       </c>
       <c r="C163" t="s">
-        <v>484</v>
+        <v>378</v>
       </c>
       <c r="D163" t="s">
-        <v>484</v>
+        <v>378</v>
       </c>
       <c r="E163" t="s">
         <v>160</v>
@@ -4357,13 +4447,13 @@
     </row>
     <row r="164" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B164" t="s">
-        <v>485</v>
+        <v>379</v>
       </c>
       <c r="C164" t="s">
-        <v>486</v>
+        <v>380</v>
       </c>
       <c r="D164" t="s">
-        <v>486</v>
+        <v>380</v>
       </c>
       <c r="E164" t="s">
         <v>160</v>
@@ -4371,13 +4461,13 @@
     </row>
     <row r="165" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B165" t="s">
-        <v>487</v>
+        <v>381</v>
       </c>
       <c r="C165" t="s">
-        <v>488</v>
+        <v>382</v>
       </c>
       <c r="D165" t="s">
-        <v>488</v>
+        <v>382</v>
       </c>
       <c r="E165" t="s">
         <v>160</v>
@@ -4385,13 +4475,13 @@
     </row>
     <row r="166" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B166" t="s">
-        <v>489</v>
+        <v>383</v>
       </c>
       <c r="C166" t="s">
-        <v>490</v>
+        <v>384</v>
       </c>
       <c r="D166" t="s">
-        <v>490</v>
+        <v>384</v>
       </c>
       <c r="E166" t="s">
         <v>160</v>
@@ -4399,13 +4489,13 @@
     </row>
     <row r="167" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B167" t="s">
-        <v>491</v>
+        <v>385</v>
       </c>
       <c r="C167" t="s">
-        <v>492</v>
+        <v>386</v>
       </c>
       <c r="D167" t="s">
-        <v>492</v>
+        <v>386</v>
       </c>
       <c r="E167" t="s">
         <v>160</v>
@@ -4651,13 +4741,13 @@
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B185" t="s">
-        <v>395</v>
+        <v>527</v>
       </c>
       <c r="C185" t="s">
-        <v>396</v>
+        <v>528</v>
       </c>
       <c r="D185" t="s">
-        <v>396</v>
+        <v>528</v>
       </c>
       <c r="E185" t="s">
         <v>160</v>
@@ -4665,13 +4755,13 @@
     </row>
     <row r="186" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B186" t="s">
-        <v>397</v>
+        <v>529</v>
       </c>
       <c r="C186" t="s">
-        <v>398</v>
+        <v>530</v>
       </c>
       <c r="D186" t="s">
-        <v>398</v>
+        <v>530</v>
       </c>
       <c r="E186" t="s">
         <v>160</v>
@@ -4679,13 +4769,13 @@
     </row>
     <row r="187" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B187" t="s">
-        <v>399</v>
+        <v>531</v>
       </c>
       <c r="C187" t="s">
-        <v>400</v>
+        <v>532</v>
       </c>
       <c r="D187" t="s">
-        <v>400</v>
+        <v>532</v>
       </c>
       <c r="E187" t="s">
         <v>160</v>
@@ -4693,13 +4783,13 @@
     </row>
     <row r="188" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B188" t="s">
-        <v>401</v>
+        <v>533</v>
       </c>
       <c r="C188" t="s">
-        <v>402</v>
+        <v>534</v>
       </c>
       <c r="D188" t="s">
-        <v>402</v>
+        <v>534</v>
       </c>
       <c r="E188" t="s">
         <v>160</v>
@@ -4707,13 +4797,13 @@
     </row>
     <row r="189" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B189" t="s">
-        <v>403</v>
+        <v>535</v>
       </c>
       <c r="C189" t="s">
-        <v>404</v>
+        <v>536</v>
       </c>
       <c r="D189" t="s">
-        <v>404</v>
+        <v>536</v>
       </c>
       <c r="E189" t="s">
         <v>160</v>
@@ -4721,13 +4811,13 @@
     </row>
     <row r="190" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B190" t="s">
-        <v>405</v>
+        <v>537</v>
       </c>
       <c r="C190" t="s">
-        <v>406</v>
+        <v>538</v>
       </c>
       <c r="D190" t="s">
-        <v>406</v>
+        <v>538</v>
       </c>
       <c r="E190" t="s">
         <v>160</v>
@@ -4735,13 +4825,13 @@
     </row>
     <row r="191" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B191" t="s">
-        <v>407</v>
+        <v>539</v>
       </c>
       <c r="C191" t="s">
-        <v>408</v>
+        <v>540</v>
       </c>
       <c r="D191" t="s">
-        <v>408</v>
+        <v>540</v>
       </c>
       <c r="E191" t="s">
         <v>160</v>
@@ -4749,13 +4839,13 @@
     </row>
     <row r="192" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B192" t="s">
-        <v>409</v>
+        <v>541</v>
       </c>
       <c r="C192" t="s">
-        <v>410</v>
+        <v>542</v>
       </c>
       <c r="D192" t="s">
-        <v>410</v>
+        <v>542</v>
       </c>
       <c r="E192" t="s">
         <v>160</v>
@@ -4763,13 +4853,13 @@
     </row>
     <row r="193" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B193" t="s">
-        <v>411</v>
+        <v>543</v>
       </c>
       <c r="C193" t="s">
-        <v>412</v>
+        <v>544</v>
       </c>
       <c r="D193" t="s">
-        <v>412</v>
+        <v>544</v>
       </c>
       <c r="E193" t="s">
         <v>160</v>
@@ -4777,15 +4867,225 @@
     </row>
     <row r="194" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B194" t="s">
-        <v>413</v>
+        <v>545</v>
       </c>
       <c r="C194" t="s">
-        <v>414</v>
+        <v>546</v>
       </c>
       <c r="D194" t="s">
-        <v>414</v>
+        <v>546</v>
       </c>
       <c r="E194" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="195" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B195" t="s">
+        <v>547</v>
+      </c>
+      <c r="C195" t="s">
+        <v>548</v>
+      </c>
+      <c r="D195" t="s">
+        <v>548</v>
+      </c>
+      <c r="E195" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="196" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B196" t="s">
+        <v>549</v>
+      </c>
+      <c r="C196" t="s">
+        <v>550</v>
+      </c>
+      <c r="D196" t="s">
+        <v>550</v>
+      </c>
+      <c r="E196" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="197" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B197" t="s">
+        <v>551</v>
+      </c>
+      <c r="C197" t="s">
+        <v>552</v>
+      </c>
+      <c r="D197" t="s">
+        <v>552</v>
+      </c>
+      <c r="E197" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="198" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B198" t="s">
+        <v>553</v>
+      </c>
+      <c r="C198" t="s">
+        <v>554</v>
+      </c>
+      <c r="D198" t="s">
+        <v>554</v>
+      </c>
+      <c r="E198" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="199" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B199" t="s">
+        <v>555</v>
+      </c>
+      <c r="C199" t="s">
+        <v>556</v>
+      </c>
+      <c r="D199" t="s">
+        <v>556</v>
+      </c>
+      <c r="E199" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="200" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B200" t="s">
+        <v>387</v>
+      </c>
+      <c r="C200" t="s">
+        <v>388</v>
+      </c>
+      <c r="D200" t="s">
+        <v>388</v>
+      </c>
+      <c r="E200" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="201" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B201" t="s">
+        <v>389</v>
+      </c>
+      <c r="C201" t="s">
+        <v>390</v>
+      </c>
+      <c r="D201" t="s">
+        <v>390</v>
+      </c>
+      <c r="E201" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="202" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B202" t="s">
+        <v>391</v>
+      </c>
+      <c r="C202" t="s">
+        <v>392</v>
+      </c>
+      <c r="D202" t="s">
+        <v>392</v>
+      </c>
+      <c r="E202" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="203" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B203" t="s">
+        <v>393</v>
+      </c>
+      <c r="C203" t="s">
+        <v>394</v>
+      </c>
+      <c r="D203" t="s">
+        <v>394</v>
+      </c>
+      <c r="E203" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="204" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B204" t="s">
+        <v>395</v>
+      </c>
+      <c r="C204" t="s">
+        <v>396</v>
+      </c>
+      <c r="D204" t="s">
+        <v>396</v>
+      </c>
+      <c r="E204" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="205" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B205" t="s">
+        <v>397</v>
+      </c>
+      <c r="C205" t="s">
+        <v>398</v>
+      </c>
+      <c r="D205" t="s">
+        <v>398</v>
+      </c>
+      <c r="E205" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="206" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B206" t="s">
+        <v>399</v>
+      </c>
+      <c r="C206" t="s">
+        <v>400</v>
+      </c>
+      <c r="D206" t="s">
+        <v>400</v>
+      </c>
+      <c r="E206" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="207" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B207" t="s">
+        <v>401</v>
+      </c>
+      <c r="C207" t="s">
+        <v>402</v>
+      </c>
+      <c r="D207" t="s">
+        <v>402</v>
+      </c>
+      <c r="E207" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="208" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B208" t="s">
+        <v>403</v>
+      </c>
+      <c r="C208" t="s">
+        <v>404</v>
+      </c>
+      <c r="D208" t="s">
+        <v>404</v>
+      </c>
+      <c r="E208" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="209" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B209" t="s">
+        <v>405</v>
+      </c>
+      <c r="C209" t="s">
+        <v>406</v>
+      </c>
+      <c r="D209" t="s">
+        <v>406</v>
+      </c>
+      <c r="E209" t="s">
         <v>160</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-19 23:21
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/Sets-vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F49DC8-A038-4969-AF13-4EE05F54EB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA89BD3-7A89-4617-9CAE-308543B67B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="515">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -616,12 +616,6 @@
     <t>*[_]Zamosc_POL</t>
   </si>
   <si>
-    <t>p_Koszalin_POL</t>
-  </si>
-  <si>
-    <t>*[_]Koszalin_POL</t>
-  </si>
-  <si>
     <t>p_Lubin_POL</t>
   </si>
   <si>
@@ -694,12 +688,6 @@
     <t>*[_]Konin_POL</t>
   </si>
   <si>
-    <t>p_Ustka_POL</t>
-  </si>
-  <si>
-    <t>*[_]Ustka_POL</t>
-  </si>
-  <si>
     <t>p_Warsaw_POL</t>
   </si>
   <si>
@@ -766,198 +754,12 @@
     <t>*[_]Gdynia_POL</t>
   </si>
   <si>
-    <t>p_Krakow_POL</t>
-  </si>
-  <si>
-    <t>*[_]Krakow_POL</t>
-  </si>
-  <si>
     <t>p_Pulawy_POL</t>
   </si>
   <si>
     <t>*[_]Pulawy_POL</t>
   </si>
   <si>
-    <t>s_ogci11072_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11072_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11074_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11074_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11075_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11075_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11076_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11076_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11077_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11077_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11078_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11078_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11079_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11079_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11080_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11080_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11081_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11081_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11082_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11082_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11083_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11083_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11084_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11084_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11085_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11085_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11086_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11086_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11087_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11087_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11088_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11088_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11089_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11089_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11090_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11090_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11091_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11091_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11092_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11092_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11093_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11093_POL</t>
-  </si>
-  <si>
-    <t>s_ogci11094_POL</t>
-  </si>
-  <si>
-    <t>*[_]ogci11094_POL</t>
-  </si>
-  <si>
-    <t>s_T1_POL</t>
-  </si>
-  <si>
-    <t>*[_]T1_POL</t>
-  </si>
-  <si>
-    <t>s_T2_POL</t>
-  </si>
-  <si>
-    <t>*[_]T2_POL</t>
-  </si>
-  <si>
-    <t>s_T3_POL</t>
-  </si>
-  <si>
-    <t>*[_]T3_POL</t>
-  </si>
-  <si>
-    <t>s_T4_POL</t>
-  </si>
-  <si>
-    <t>*[_]T4_POL</t>
-  </si>
-  <si>
-    <t>s_T5_POL</t>
-  </si>
-  <si>
-    <t>*[_]T5_POL</t>
-  </si>
-  <si>
-    <t>s_T6_POL</t>
-  </si>
-  <si>
-    <t>*[_]T6_POL</t>
-  </si>
-  <si>
-    <t>s_T7_POL</t>
-  </si>
-  <si>
-    <t>*[_]T7_POL</t>
-  </si>
-  <si>
-    <t>s_T8_POL</t>
-  </si>
-  <si>
-    <t>*[_]T8_POL</t>
-  </si>
-  <si>
     <t>rez_spv_POL_001</t>
   </si>
   <si>
@@ -1270,12 +1072,6 @@
     <t>*[_]Lukow_POL</t>
   </si>
   <si>
-    <t>p_Ostroleka_POL</t>
-  </si>
-  <si>
-    <t>*[_]Ostroleka_POL</t>
-  </si>
-  <si>
     <t>p_Lublin_POL</t>
   </si>
   <si>
@@ -1288,6 +1084,12 @@
     <t>*[_]Radom_POL</t>
   </si>
   <si>
+    <t>p_Skawina_POL</t>
+  </si>
+  <si>
+    <t>*[_]Skawina_POL</t>
+  </si>
+  <si>
     <t>p_Pila_POL</t>
   </si>
   <si>
@@ -1312,12 +1114,114 @@
     <t>*[_]Belchatow_POL</t>
   </si>
   <si>
+    <t>p_Zabrze_POL</t>
+  </si>
+  <si>
+    <t>*[_]Zabrze_POL</t>
+  </si>
+  <si>
     <t>p_Lodz_POL</t>
   </si>
   <si>
     <t>*[_]Lodz_POL</t>
   </si>
   <si>
+    <t>s_PGI005_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI005_POL</t>
+  </si>
+  <si>
+    <t>s_PGI038_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI038_POL</t>
+  </si>
+  <si>
+    <t>s_PGI011_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI011_POL</t>
+  </si>
+  <si>
+    <t>s_PGI014_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI014_POL</t>
+  </si>
+  <si>
+    <t>s_PGI015_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI015_POL</t>
+  </si>
+  <si>
+    <t>s_PGI013_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI013_POL</t>
+  </si>
+  <si>
+    <t>s_PGI003_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI003_POL</t>
+  </si>
+  <si>
+    <t>s_PGI020_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI020_POL</t>
+  </si>
+  <si>
+    <t>s_PGI012_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI012_POL</t>
+  </si>
+  <si>
+    <t>s_PGI019_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI019_POL</t>
+  </si>
+  <si>
+    <t>s_PGI016_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI016_POL</t>
+  </si>
+  <si>
+    <t>s_PGI032_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI032_POL</t>
+  </si>
+  <si>
+    <t>s_PGI035_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI035_POL</t>
+  </si>
+  <si>
+    <t>s_PGI033_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI033_POL</t>
+  </si>
+  <si>
+    <t>s_PGI027_POL</t>
+  </si>
+  <si>
+    <t>*[_]PGI027_POL</t>
+  </si>
+  <si>
+    <t>s_ExportNL_POL</t>
+  </si>
+  <si>
+    <t>*[_]ExportNL_POL</t>
+  </si>
+  <si>
     <t>rez_spv_POL_021</t>
   </si>
   <si>
@@ -1504,18 +1408,6 @@
     <t>elc_spv_POL_051</t>
   </si>
   <si>
-    <t>rez_spv_POL_052</t>
-  </si>
-  <si>
-    <t>elc_spv_POL_052</t>
-  </si>
-  <si>
-    <t>rez_spv_POL_053</t>
-  </si>
-  <si>
-    <t>elc_spv_POL_053</t>
-  </si>
-  <si>
     <t>rez_won_POL_021</t>
   </si>
   <si>
@@ -1688,24 +1580,6 @@
   </si>
   <si>
     <t>elc_won_POL_049</t>
-  </si>
-  <si>
-    <t>rez_won_POL_050</t>
-  </si>
-  <si>
-    <t>elc_won_POL_050</t>
-  </si>
-  <si>
-    <t>rez_won_POL_051</t>
-  </si>
-  <si>
-    <t>elc_won_POL_051</t>
-  </si>
-  <si>
-    <t>rez_won_POL_052</t>
-  </si>
-  <si>
-    <t>elc_won_POL_052</t>
   </si>
 </sst>
 </file>
@@ -2281,7 +2155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B9:E209"/>
+  <dimension ref="B9:E188"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -2347,13 +2221,13 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>407</v>
+        <v>341</v>
       </c>
       <c r="C14" t="s">
-        <v>408</v>
+        <v>342</v>
       </c>
       <c r="D14" t="s">
-        <v>408</v>
+        <v>342</v>
       </c>
       <c r="E14" t="s">
         <v>160</v>
@@ -2361,13 +2235,13 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>409</v>
+        <v>343</v>
       </c>
       <c r="C15" t="s">
-        <v>410</v>
+        <v>344</v>
       </c>
       <c r="D15" t="s">
-        <v>410</v>
+        <v>344</v>
       </c>
       <c r="E15" t="s">
         <v>160</v>
@@ -2487,13 +2361,13 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>411</v>
+        <v>179</v>
       </c>
       <c r="C24" t="s">
-        <v>412</v>
+        <v>180</v>
       </c>
       <c r="D24" t="s">
-        <v>412</v>
+        <v>180</v>
       </c>
       <c r="E24" t="s">
         <v>160</v>
@@ -2501,13 +2375,13 @@
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C25" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D25" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E25" t="s">
         <v>160</v>
@@ -2515,13 +2389,13 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C26" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D26" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E26" t="s">
         <v>160</v>
@@ -2529,13 +2403,13 @@
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>183</v>
+        <v>345</v>
       </c>
       <c r="C27" t="s">
-        <v>184</v>
+        <v>346</v>
       </c>
       <c r="D27" t="s">
-        <v>184</v>
+        <v>346</v>
       </c>
       <c r="E27" t="s">
         <v>160</v>
@@ -2543,13 +2417,13 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>413</v>
+        <v>187</v>
       </c>
       <c r="C28" t="s">
-        <v>414</v>
+        <v>188</v>
       </c>
       <c r="D28" t="s">
-        <v>414</v>
+        <v>188</v>
       </c>
       <c r="E28" t="s">
         <v>160</v>
@@ -2557,13 +2431,13 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C29" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D29" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E29" t="s">
         <v>160</v>
@@ -2571,13 +2445,13 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E30" t="s">
         <v>160</v>
@@ -2585,13 +2459,13 @@
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>189</v>
+        <v>347</v>
       </c>
       <c r="C31" t="s">
-        <v>190</v>
+        <v>348</v>
       </c>
       <c r="D31" t="s">
-        <v>190</v>
+        <v>348</v>
       </c>
       <c r="E31" t="s">
         <v>160</v>
@@ -2599,13 +2473,13 @@
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>415</v>
+        <v>193</v>
       </c>
       <c r="C32" t="s">
-        <v>416</v>
+        <v>194</v>
       </c>
       <c r="D32" t="s">
-        <v>416</v>
+        <v>194</v>
       </c>
       <c r="E32" t="s">
         <v>160</v>
@@ -2613,13 +2487,13 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C33" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D33" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E33" t="s">
         <v>160</v>
@@ -2627,13 +2501,13 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
-        <v>195</v>
+        <v>349</v>
       </c>
       <c r="C34" t="s">
-        <v>196</v>
+        <v>350</v>
       </c>
       <c r="D34" t="s">
-        <v>196</v>
+        <v>350</v>
       </c>
       <c r="E34" t="s">
         <v>160</v>
@@ -2725,13 +2599,13 @@
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" t="s">
-        <v>209</v>
+        <v>351</v>
       </c>
       <c r="C41" t="s">
-        <v>210</v>
+        <v>352</v>
       </c>
       <c r="D41" t="s">
-        <v>210</v>
+        <v>352</v>
       </c>
       <c r="E41" t="s">
         <v>160</v>
@@ -2739,13 +2613,13 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" t="s">
-        <v>417</v>
+        <v>211</v>
       </c>
       <c r="C42" t="s">
-        <v>418</v>
+        <v>212</v>
       </c>
       <c r="D42" t="s">
-        <v>418</v>
+        <v>212</v>
       </c>
       <c r="E42" t="s">
         <v>160</v>
@@ -2753,13 +2627,13 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C43" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D43" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E43" t="s">
         <v>160</v>
@@ -2767,13 +2641,13 @@
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C44" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D44" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E44" t="s">
         <v>160</v>
@@ -2781,13 +2655,13 @@
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" t="s">
-        <v>215</v>
+        <v>353</v>
       </c>
       <c r="C45" t="s">
-        <v>216</v>
+        <v>354</v>
       </c>
       <c r="D45" t="s">
-        <v>216</v>
+        <v>354</v>
       </c>
       <c r="E45" t="s">
         <v>160</v>
@@ -2795,13 +2669,13 @@
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" t="s">
-        <v>217</v>
+        <v>355</v>
       </c>
       <c r="C46" t="s">
-        <v>218</v>
+        <v>356</v>
       </c>
       <c r="D46" t="s">
-        <v>218</v>
+        <v>356</v>
       </c>
       <c r="E46" t="s">
         <v>160</v>
@@ -2809,13 +2683,13 @@
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" t="s">
-        <v>419</v>
+        <v>217</v>
       </c>
       <c r="C47" t="s">
-        <v>420</v>
+        <v>218</v>
       </c>
       <c r="D47" t="s">
-        <v>420</v>
+        <v>218</v>
       </c>
       <c r="E47" t="s">
         <v>160</v>
@@ -2823,13 +2697,13 @@
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
-        <v>219</v>
+        <v>357</v>
       </c>
       <c r="C48" t="s">
-        <v>220</v>
+        <v>358</v>
       </c>
       <c r="D48" t="s">
-        <v>220</v>
+        <v>358</v>
       </c>
       <c r="E48" t="s">
         <v>160</v>
@@ -2837,13 +2711,13 @@
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" t="s">
-        <v>421</v>
+        <v>359</v>
       </c>
       <c r="C49" t="s">
-        <v>422</v>
+        <v>360</v>
       </c>
       <c r="D49" t="s">
-        <v>422</v>
+        <v>360</v>
       </c>
       <c r="E49" t="s">
         <v>160</v>
@@ -2851,13 +2725,13 @@
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C50" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D50" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E50" t="s">
         <v>160</v>
@@ -2865,13 +2739,13 @@
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" t="s">
-        <v>423</v>
+        <v>221</v>
       </c>
       <c r="C51" t="s">
-        <v>424</v>
+        <v>222</v>
       </c>
       <c r="D51" t="s">
-        <v>424</v>
+        <v>222</v>
       </c>
       <c r="E51" t="s">
         <v>160</v>
@@ -2893,13 +2767,13 @@
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B53" t="s">
-        <v>225</v>
+        <v>361</v>
       </c>
       <c r="C53" t="s">
-        <v>226</v>
+        <v>362</v>
       </c>
       <c r="D53" t="s">
-        <v>226</v>
+        <v>362</v>
       </c>
       <c r="E53" t="s">
         <v>160</v>
@@ -2907,13 +2781,13 @@
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B54" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C54" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D54" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E54" t="s">
         <v>160</v>
@@ -2921,13 +2795,13 @@
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B55" t="s">
-        <v>425</v>
+        <v>227</v>
       </c>
       <c r="C55" t="s">
-        <v>426</v>
+        <v>228</v>
       </c>
       <c r="D55" t="s">
-        <v>426</v>
+        <v>228</v>
       </c>
       <c r="E55" t="s">
         <v>160</v>
@@ -2977,13 +2851,13 @@
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B59" t="s">
-        <v>235</v>
+        <v>209</v>
       </c>
       <c r="C59" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="D59" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="E59" t="s">
         <v>160</v>
@@ -2991,13 +2865,13 @@
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B60" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C60" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D60" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E60" t="s">
         <v>160</v>
@@ -3005,13 +2879,13 @@
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B61" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C61" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D61" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E61" t="s">
         <v>160</v>
@@ -3019,13 +2893,13 @@
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B62" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C62" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D62" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E62" t="s">
         <v>160</v>
@@ -3033,13 +2907,13 @@
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B63" t="s">
-        <v>243</v>
+        <v>363</v>
       </c>
       <c r="C63" t="s">
-        <v>244</v>
+        <v>364</v>
       </c>
       <c r="D63" t="s">
-        <v>244</v>
+        <v>364</v>
       </c>
       <c r="E63" t="s">
         <v>160</v>
@@ -3047,13 +2921,13 @@
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B64" t="s">
-        <v>245</v>
+        <v>365</v>
       </c>
       <c r="C64" t="s">
-        <v>246</v>
+        <v>366</v>
       </c>
       <c r="D64" t="s">
-        <v>246</v>
+        <v>366</v>
       </c>
       <c r="E64" t="s">
         <v>160</v>
@@ -3061,13 +2935,13 @@
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B65" t="s">
-        <v>247</v>
+        <v>367</v>
       </c>
       <c r="C65" t="s">
-        <v>248</v>
+        <v>368</v>
       </c>
       <c r="D65" t="s">
-        <v>248</v>
+        <v>368</v>
       </c>
       <c r="E65" t="s">
         <v>160</v>
@@ -3075,13 +2949,13 @@
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B66" t="s">
-        <v>249</v>
+        <v>369</v>
       </c>
       <c r="C66" t="s">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="D66" t="s">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="E66" t="s">
         <v>160</v>
@@ -3089,13 +2963,13 @@
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B67" t="s">
-        <v>251</v>
+        <v>371</v>
       </c>
       <c r="C67" t="s">
-        <v>252</v>
+        <v>372</v>
       </c>
       <c r="D67" t="s">
-        <v>252</v>
+        <v>372</v>
       </c>
       <c r="E67" t="s">
         <v>160</v>
@@ -3103,13 +2977,13 @@
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B68" t="s">
-        <v>253</v>
+        <v>373</v>
       </c>
       <c r="C68" t="s">
-        <v>254</v>
+        <v>374</v>
       </c>
       <c r="D68" t="s">
-        <v>254</v>
+        <v>374</v>
       </c>
       <c r="E68" t="s">
         <v>160</v>
@@ -3117,13 +2991,13 @@
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B69" t="s">
-        <v>255</v>
+        <v>375</v>
       </c>
       <c r="C69" t="s">
-        <v>256</v>
+        <v>376</v>
       </c>
       <c r="D69" t="s">
-        <v>256</v>
+        <v>376</v>
       </c>
       <c r="E69" t="s">
         <v>160</v>
@@ -3131,13 +3005,13 @@
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B70" t="s">
-        <v>257</v>
+        <v>377</v>
       </c>
       <c r="C70" t="s">
-        <v>258</v>
+        <v>378</v>
       </c>
       <c r="D70" t="s">
-        <v>258</v>
+        <v>378</v>
       </c>
       <c r="E70" t="s">
         <v>160</v>
@@ -3145,13 +3019,13 @@
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B71" t="s">
-        <v>259</v>
+        <v>379</v>
       </c>
       <c r="C71" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="D71" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="E71" t="s">
         <v>160</v>
@@ -3159,13 +3033,13 @@
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B72" t="s">
-        <v>261</v>
+        <v>381</v>
       </c>
       <c r="C72" t="s">
-        <v>262</v>
+        <v>382</v>
       </c>
       <c r="D72" t="s">
-        <v>262</v>
+        <v>382</v>
       </c>
       <c r="E72" t="s">
         <v>160</v>
@@ -3173,13 +3047,13 @@
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B73" t="s">
-        <v>263</v>
+        <v>383</v>
       </c>
       <c r="C73" t="s">
-        <v>264</v>
+        <v>384</v>
       </c>
       <c r="D73" t="s">
-        <v>264</v>
+        <v>384</v>
       </c>
       <c r="E73" t="s">
         <v>160</v>
@@ -3187,13 +3061,13 @@
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B74" t="s">
-        <v>265</v>
+        <v>385</v>
       </c>
       <c r="C74" t="s">
-        <v>266</v>
+        <v>386</v>
       </c>
       <c r="D74" t="s">
-        <v>266</v>
+        <v>386</v>
       </c>
       <c r="E74" t="s">
         <v>160</v>
@@ -3201,13 +3075,13 @@
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B75" t="s">
-        <v>267</v>
+        <v>387</v>
       </c>
       <c r="C75" t="s">
-        <v>268</v>
+        <v>388</v>
       </c>
       <c r="D75" t="s">
-        <v>268</v>
+        <v>388</v>
       </c>
       <c r="E75" t="s">
         <v>160</v>
@@ -3215,13 +3089,13 @@
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B76" t="s">
-        <v>269</v>
+        <v>389</v>
       </c>
       <c r="C76" t="s">
-        <v>270</v>
+        <v>390</v>
       </c>
       <c r="D76" t="s">
-        <v>270</v>
+        <v>390</v>
       </c>
       <c r="E76" t="s">
         <v>160</v>
@@ -3229,13 +3103,13 @@
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B77" t="s">
-        <v>271</v>
+        <v>391</v>
       </c>
       <c r="C77" t="s">
-        <v>272</v>
+        <v>392</v>
       </c>
       <c r="D77" t="s">
-        <v>272</v>
+        <v>392</v>
       </c>
       <c r="E77" t="s">
         <v>160</v>
@@ -3243,13 +3117,13 @@
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B78" t="s">
-        <v>273</v>
+        <v>393</v>
       </c>
       <c r="C78" t="s">
-        <v>274</v>
+        <v>394</v>
       </c>
       <c r="D78" t="s">
-        <v>274</v>
+        <v>394</v>
       </c>
       <c r="E78" t="s">
         <v>160</v>
@@ -3257,13 +3131,13 @@
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B79" t="s">
-        <v>275</v>
+        <v>241</v>
       </c>
       <c r="C79" t="s">
-        <v>276</v>
+        <v>242</v>
       </c>
       <c r="D79" t="s">
-        <v>276</v>
+        <v>242</v>
       </c>
       <c r="E79" t="s">
         <v>160</v>
@@ -3271,13 +3145,13 @@
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B80" t="s">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="C80" t="s">
-        <v>278</v>
+        <v>244</v>
       </c>
       <c r="D80" t="s">
-        <v>278</v>
+        <v>244</v>
       </c>
       <c r="E80" t="s">
         <v>160</v>
@@ -3285,13 +3159,13 @@
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B81" t="s">
-        <v>279</v>
+        <v>245</v>
       </c>
       <c r="C81" t="s">
-        <v>280</v>
+        <v>246</v>
       </c>
       <c r="D81" t="s">
-        <v>280</v>
+        <v>246</v>
       </c>
       <c r="E81" t="s">
         <v>160</v>
@@ -3299,13 +3173,13 @@
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B82" t="s">
-        <v>281</v>
+        <v>247</v>
       </c>
       <c r="C82" t="s">
-        <v>282</v>
+        <v>248</v>
       </c>
       <c r="D82" t="s">
-        <v>282</v>
+        <v>248</v>
       </c>
       <c r="E82" t="s">
         <v>160</v>
@@ -3313,13 +3187,13 @@
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B83" t="s">
-        <v>283</v>
+        <v>249</v>
       </c>
       <c r="C83" t="s">
-        <v>284</v>
+        <v>250</v>
       </c>
       <c r="D83" t="s">
-        <v>284</v>
+        <v>250</v>
       </c>
       <c r="E83" t="s">
         <v>160</v>
@@ -3327,13 +3201,13 @@
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B84" t="s">
-        <v>285</v>
+        <v>251</v>
       </c>
       <c r="C84" t="s">
-        <v>286</v>
+        <v>252</v>
       </c>
       <c r="D84" t="s">
-        <v>286</v>
+        <v>252</v>
       </c>
       <c r="E84" t="s">
         <v>160</v>
@@ -3341,13 +3215,13 @@
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B85" t="s">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="C85" t="s">
-        <v>288</v>
+        <v>254</v>
       </c>
       <c r="D85" t="s">
-        <v>288</v>
+        <v>254</v>
       </c>
       <c r="E85" t="s">
         <v>160</v>
@@ -3355,13 +3229,13 @@
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B86" t="s">
-        <v>289</v>
+        <v>255</v>
       </c>
       <c r="C86" t="s">
-        <v>290</v>
+        <v>256</v>
       </c>
       <c r="D86" t="s">
-        <v>290</v>
+        <v>256</v>
       </c>
       <c r="E86" t="s">
         <v>160</v>
@@ -3369,13 +3243,13 @@
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B87" t="s">
-        <v>291</v>
+        <v>257</v>
       </c>
       <c r="C87" t="s">
-        <v>292</v>
+        <v>258</v>
       </c>
       <c r="D87" t="s">
-        <v>292</v>
+        <v>258</v>
       </c>
       <c r="E87" t="s">
         <v>160</v>
@@ -3383,13 +3257,13 @@
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B88" t="s">
-        <v>293</v>
+        <v>259</v>
       </c>
       <c r="C88" t="s">
-        <v>294</v>
+        <v>260</v>
       </c>
       <c r="D88" t="s">
-        <v>294</v>
+        <v>260</v>
       </c>
       <c r="E88" t="s">
         <v>160</v>
@@ -3397,13 +3271,13 @@
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B89" t="s">
-        <v>295</v>
+        <v>261</v>
       </c>
       <c r="C89" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="D89" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="E89" t="s">
         <v>160</v>
@@ -3411,13 +3285,13 @@
     </row>
     <row r="90" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B90" t="s">
-        <v>297</v>
+        <v>263</v>
       </c>
       <c r="C90" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="D90" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="E90" t="s">
         <v>160</v>
@@ -3425,13 +3299,13 @@
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B91" t="s">
-        <v>299</v>
+        <v>265</v>
       </c>
       <c r="C91" t="s">
-        <v>300</v>
+        <v>266</v>
       </c>
       <c r="D91" t="s">
-        <v>300</v>
+        <v>266</v>
       </c>
       <c r="E91" t="s">
         <v>160</v>
@@ -3439,13 +3313,13 @@
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B92" t="s">
-        <v>301</v>
+        <v>267</v>
       </c>
       <c r="C92" t="s">
-        <v>302</v>
+        <v>268</v>
       </c>
       <c r="D92" t="s">
-        <v>302</v>
+        <v>268</v>
       </c>
       <c r="E92" t="s">
         <v>160</v>
@@ -3453,13 +3327,13 @@
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B93" t="s">
-        <v>303</v>
+        <v>269</v>
       </c>
       <c r="C93" t="s">
-        <v>304</v>
+        <v>270</v>
       </c>
       <c r="D93" t="s">
-        <v>304</v>
+        <v>270</v>
       </c>
       <c r="E93" t="s">
         <v>160</v>
@@ -3467,13 +3341,13 @@
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B94" t="s">
-        <v>305</v>
+        <v>271</v>
       </c>
       <c r="C94" t="s">
-        <v>306</v>
+        <v>272</v>
       </c>
       <c r="D94" t="s">
-        <v>306</v>
+        <v>272</v>
       </c>
       <c r="E94" t="s">
         <v>160</v>
@@ -3481,13 +3355,13 @@
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B95" t="s">
-        <v>307</v>
+        <v>273</v>
       </c>
       <c r="C95" t="s">
-        <v>308</v>
+        <v>274</v>
       </c>
       <c r="D95" t="s">
-        <v>308</v>
+        <v>274</v>
       </c>
       <c r="E95" t="s">
         <v>160</v>
@@ -3495,13 +3369,13 @@
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B96" t="s">
-        <v>309</v>
+        <v>275</v>
       </c>
       <c r="C96" t="s">
-        <v>310</v>
+        <v>276</v>
       </c>
       <c r="D96" t="s">
-        <v>310</v>
+        <v>276</v>
       </c>
       <c r="E96" t="s">
         <v>160</v>
@@ -3509,13 +3383,13 @@
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B97" t="s">
-        <v>311</v>
+        <v>277</v>
       </c>
       <c r="C97" t="s">
-        <v>312</v>
+        <v>278</v>
       </c>
       <c r="D97" t="s">
-        <v>312</v>
+        <v>278</v>
       </c>
       <c r="E97" t="s">
         <v>160</v>
@@ -3523,13 +3397,13 @@
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B98" t="s">
-        <v>313</v>
+        <v>279</v>
       </c>
       <c r="C98" t="s">
-        <v>314</v>
+        <v>280</v>
       </c>
       <c r="D98" t="s">
-        <v>314</v>
+        <v>280</v>
       </c>
       <c r="E98" t="s">
         <v>160</v>
@@ -3537,13 +3411,13 @@
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B99" t="s">
-        <v>315</v>
+        <v>395</v>
       </c>
       <c r="C99" t="s">
-        <v>316</v>
+        <v>396</v>
       </c>
       <c r="D99" t="s">
-        <v>316</v>
+        <v>396</v>
       </c>
       <c r="E99" t="s">
         <v>160</v>
@@ -3551,13 +3425,13 @@
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B100" t="s">
-        <v>317</v>
+        <v>397</v>
       </c>
       <c r="C100" t="s">
-        <v>318</v>
+        <v>398</v>
       </c>
       <c r="D100" t="s">
-        <v>318</v>
+        <v>398</v>
       </c>
       <c r="E100" t="s">
         <v>160</v>
@@ -3565,13 +3439,13 @@
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B101" t="s">
-        <v>319</v>
+        <v>399</v>
       </c>
       <c r="C101" t="s">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="D101" t="s">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="E101" t="s">
         <v>160</v>
@@ -3579,13 +3453,13 @@
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B102" t="s">
-        <v>321</v>
+        <v>401</v>
       </c>
       <c r="C102" t="s">
-        <v>322</v>
+        <v>402</v>
       </c>
       <c r="D102" t="s">
-        <v>322</v>
+        <v>402</v>
       </c>
       <c r="E102" t="s">
         <v>160</v>
@@ -3593,13 +3467,13 @@
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B103" t="s">
-        <v>323</v>
+        <v>403</v>
       </c>
       <c r="C103" t="s">
-        <v>324</v>
+        <v>404</v>
       </c>
       <c r="D103" t="s">
-        <v>324</v>
+        <v>404</v>
       </c>
       <c r="E103" t="s">
         <v>160</v>
@@ -3607,13 +3481,13 @@
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B104" t="s">
-        <v>325</v>
+        <v>405</v>
       </c>
       <c r="C104" t="s">
-        <v>326</v>
+        <v>406</v>
       </c>
       <c r="D104" t="s">
-        <v>326</v>
+        <v>406</v>
       </c>
       <c r="E104" t="s">
         <v>160</v>
@@ -3621,13 +3495,13 @@
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B105" t="s">
-        <v>327</v>
+        <v>407</v>
       </c>
       <c r="C105" t="s">
-        <v>328</v>
+        <v>408</v>
       </c>
       <c r="D105" t="s">
-        <v>328</v>
+        <v>408</v>
       </c>
       <c r="E105" t="s">
         <v>160</v>
@@ -3635,13 +3509,13 @@
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B106" t="s">
-        <v>329</v>
+        <v>409</v>
       </c>
       <c r="C106" t="s">
-        <v>330</v>
+        <v>410</v>
       </c>
       <c r="D106" t="s">
-        <v>330</v>
+        <v>410</v>
       </c>
       <c r="E106" t="s">
         <v>160</v>
@@ -3649,13 +3523,13 @@
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B107" t="s">
-        <v>331</v>
+        <v>411</v>
       </c>
       <c r="C107" t="s">
-        <v>332</v>
+        <v>412</v>
       </c>
       <c r="D107" t="s">
-        <v>332</v>
+        <v>412</v>
       </c>
       <c r="E107" t="s">
         <v>160</v>
@@ -3663,13 +3537,13 @@
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B108" t="s">
-        <v>333</v>
+        <v>413</v>
       </c>
       <c r="C108" t="s">
-        <v>334</v>
+        <v>414</v>
       </c>
       <c r="D108" t="s">
-        <v>334</v>
+        <v>414</v>
       </c>
       <c r="E108" t="s">
         <v>160</v>
@@ -3677,13 +3551,13 @@
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B109" t="s">
-        <v>335</v>
+        <v>415</v>
       </c>
       <c r="C109" t="s">
-        <v>336</v>
+        <v>416</v>
       </c>
       <c r="D109" t="s">
-        <v>336</v>
+        <v>416</v>
       </c>
       <c r="E109" t="s">
         <v>160</v>
@@ -3691,13 +3565,13 @@
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B110" t="s">
-        <v>337</v>
+        <v>417</v>
       </c>
       <c r="C110" t="s">
-        <v>338</v>
+        <v>418</v>
       </c>
       <c r="D110" t="s">
-        <v>338</v>
+        <v>418</v>
       </c>
       <c r="E110" t="s">
         <v>160</v>
@@ -3705,13 +3579,13 @@
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B111" t="s">
-        <v>339</v>
+        <v>419</v>
       </c>
       <c r="C111" t="s">
-        <v>340</v>
+        <v>420</v>
       </c>
       <c r="D111" t="s">
-        <v>340</v>
+        <v>420</v>
       </c>
       <c r="E111" t="s">
         <v>160</v>
@@ -3719,13 +3593,13 @@
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B112" t="s">
-        <v>341</v>
+        <v>421</v>
       </c>
       <c r="C112" t="s">
-        <v>342</v>
+        <v>422</v>
       </c>
       <c r="D112" t="s">
-        <v>342</v>
+        <v>422</v>
       </c>
       <c r="E112" t="s">
         <v>160</v>
@@ -3733,13 +3607,13 @@
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B113" t="s">
-        <v>343</v>
+        <v>423</v>
       </c>
       <c r="C113" t="s">
-        <v>344</v>
+        <v>424</v>
       </c>
       <c r="D113" t="s">
-        <v>344</v>
+        <v>424</v>
       </c>
       <c r="E113" t="s">
         <v>160</v>
@@ -3747,13 +3621,13 @@
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B114" t="s">
-        <v>345</v>
+        <v>425</v>
       </c>
       <c r="C114" t="s">
-        <v>346</v>
+        <v>426</v>
       </c>
       <c r="D114" t="s">
-        <v>346</v>
+        <v>426</v>
       </c>
       <c r="E114" t="s">
         <v>160</v>
@@ -3971,13 +3845,13 @@
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B130" t="s">
-        <v>457</v>
+        <v>281</v>
       </c>
       <c r="C130" t="s">
-        <v>458</v>
+        <v>282</v>
       </c>
       <c r="D130" t="s">
-        <v>458</v>
+        <v>282</v>
       </c>
       <c r="E130" t="s">
         <v>160</v>
@@ -3985,13 +3859,13 @@
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B131" t="s">
-        <v>459</v>
+        <v>283</v>
       </c>
       <c r="C131" t="s">
-        <v>460</v>
+        <v>284</v>
       </c>
       <c r="D131" t="s">
-        <v>460</v>
+        <v>284</v>
       </c>
       <c r="E131" t="s">
         <v>160</v>
@@ -3999,13 +3873,13 @@
     </row>
     <row r="132" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B132" t="s">
-        <v>461</v>
+        <v>285</v>
       </c>
       <c r="C132" t="s">
-        <v>462</v>
+        <v>286</v>
       </c>
       <c r="D132" t="s">
-        <v>462</v>
+        <v>286</v>
       </c>
       <c r="E132" t="s">
         <v>160</v>
@@ -4013,13 +3887,13 @@
     </row>
     <row r="133" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B133" t="s">
-        <v>463</v>
+        <v>287</v>
       </c>
       <c r="C133" t="s">
-        <v>464</v>
+        <v>288</v>
       </c>
       <c r="D133" t="s">
-        <v>464</v>
+        <v>288</v>
       </c>
       <c r="E133" t="s">
         <v>160</v>
@@ -4027,13 +3901,13 @@
     </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B134" t="s">
-        <v>465</v>
+        <v>289</v>
       </c>
       <c r="C134" t="s">
-        <v>466</v>
+        <v>290</v>
       </c>
       <c r="D134" t="s">
-        <v>466</v>
+        <v>290</v>
       </c>
       <c r="E134" t="s">
         <v>160</v>
@@ -4041,13 +3915,13 @@
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B135" t="s">
-        <v>467</v>
+        <v>291</v>
       </c>
       <c r="C135" t="s">
-        <v>468</v>
+        <v>292</v>
       </c>
       <c r="D135" t="s">
-        <v>468</v>
+        <v>292</v>
       </c>
       <c r="E135" t="s">
         <v>160</v>
@@ -4055,13 +3929,13 @@
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B136" t="s">
-        <v>469</v>
+        <v>293</v>
       </c>
       <c r="C136" t="s">
-        <v>470</v>
+        <v>294</v>
       </c>
       <c r="D136" t="s">
-        <v>470</v>
+        <v>294</v>
       </c>
       <c r="E136" t="s">
         <v>160</v>
@@ -4069,13 +3943,13 @@
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B137" t="s">
-        <v>471</v>
+        <v>295</v>
       </c>
       <c r="C137" t="s">
-        <v>472</v>
+        <v>296</v>
       </c>
       <c r="D137" t="s">
-        <v>472</v>
+        <v>296</v>
       </c>
       <c r="E137" t="s">
         <v>160</v>
@@ -4083,13 +3957,13 @@
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B138" t="s">
-        <v>473</v>
+        <v>297</v>
       </c>
       <c r="C138" t="s">
-        <v>474</v>
+        <v>298</v>
       </c>
       <c r="D138" t="s">
-        <v>474</v>
+        <v>298</v>
       </c>
       <c r="E138" t="s">
         <v>160</v>
@@ -4097,13 +3971,13 @@
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B139" t="s">
-        <v>475</v>
+        <v>299</v>
       </c>
       <c r="C139" t="s">
-        <v>476</v>
+        <v>300</v>
       </c>
       <c r="D139" t="s">
-        <v>476</v>
+        <v>300</v>
       </c>
       <c r="E139" t="s">
         <v>160</v>
@@ -4111,13 +3985,13 @@
     </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B140" t="s">
-        <v>477</v>
+        <v>301</v>
       </c>
       <c r="C140" t="s">
-        <v>478</v>
+        <v>302</v>
       </c>
       <c r="D140" t="s">
-        <v>478</v>
+        <v>302</v>
       </c>
       <c r="E140" t="s">
         <v>160</v>
@@ -4125,13 +3999,13 @@
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B141" t="s">
-        <v>479</v>
+        <v>303</v>
       </c>
       <c r="C141" t="s">
-        <v>480</v>
+        <v>304</v>
       </c>
       <c r="D141" t="s">
-        <v>480</v>
+        <v>304</v>
       </c>
       <c r="E141" t="s">
         <v>160</v>
@@ -4139,13 +4013,13 @@
     </row>
     <row r="142" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B142" t="s">
-        <v>481</v>
+        <v>305</v>
       </c>
       <c r="C142" t="s">
-        <v>482</v>
+        <v>306</v>
       </c>
       <c r="D142" t="s">
-        <v>482</v>
+        <v>306</v>
       </c>
       <c r="E142" t="s">
         <v>160</v>
@@ -4153,13 +4027,13 @@
     </row>
     <row r="143" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B143" t="s">
-        <v>483</v>
+        <v>307</v>
       </c>
       <c r="C143" t="s">
-        <v>484</v>
+        <v>308</v>
       </c>
       <c r="D143" t="s">
-        <v>484</v>
+        <v>308</v>
       </c>
       <c r="E143" t="s">
         <v>160</v>
@@ -4167,13 +4041,13 @@
     </row>
     <row r="144" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B144" t="s">
-        <v>485</v>
+        <v>309</v>
       </c>
       <c r="C144" t="s">
-        <v>486</v>
+        <v>310</v>
       </c>
       <c r="D144" t="s">
-        <v>486</v>
+        <v>310</v>
       </c>
       <c r="E144" t="s">
         <v>160</v>
@@ -4181,13 +4055,13 @@
     </row>
     <row r="145" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B145" t="s">
-        <v>487</v>
+        <v>311</v>
       </c>
       <c r="C145" t="s">
-        <v>488</v>
+        <v>312</v>
       </c>
       <c r="D145" t="s">
-        <v>488</v>
+        <v>312</v>
       </c>
       <c r="E145" t="s">
         <v>160</v>
@@ -4195,13 +4069,13 @@
     </row>
     <row r="146" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B146" t="s">
-        <v>489</v>
+        <v>313</v>
       </c>
       <c r="C146" t="s">
-        <v>490</v>
+        <v>314</v>
       </c>
       <c r="D146" t="s">
-        <v>490</v>
+        <v>314</v>
       </c>
       <c r="E146" t="s">
         <v>160</v>
@@ -4209,13 +4083,13 @@
     </row>
     <row r="147" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B147" t="s">
-        <v>491</v>
+        <v>315</v>
       </c>
       <c r="C147" t="s">
-        <v>492</v>
+        <v>316</v>
       </c>
       <c r="D147" t="s">
-        <v>492</v>
+        <v>316</v>
       </c>
       <c r="E147" t="s">
         <v>160</v>
@@ -4223,13 +4097,13 @@
     </row>
     <row r="148" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B148" t="s">
-        <v>347</v>
+        <v>317</v>
       </c>
       <c r="C148" t="s">
-        <v>348</v>
+        <v>318</v>
       </c>
       <c r="D148" t="s">
-        <v>348</v>
+        <v>318</v>
       </c>
       <c r="E148" t="s">
         <v>160</v>
@@ -4237,13 +4111,13 @@
     </row>
     <row r="149" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B149" t="s">
-        <v>349</v>
+        <v>319</v>
       </c>
       <c r="C149" t="s">
-        <v>350</v>
+        <v>320</v>
       </c>
       <c r="D149" t="s">
-        <v>350</v>
+        <v>320</v>
       </c>
       <c r="E149" t="s">
         <v>160</v>
@@ -4251,13 +4125,13 @@
     </row>
     <row r="150" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B150" t="s">
-        <v>351</v>
+        <v>457</v>
       </c>
       <c r="C150" t="s">
-        <v>352</v>
+        <v>458</v>
       </c>
       <c r="D150" t="s">
-        <v>352</v>
+        <v>458</v>
       </c>
       <c r="E150" t="s">
         <v>160</v>
@@ -4265,13 +4139,13 @@
     </row>
     <row r="151" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B151" t="s">
-        <v>353</v>
+        <v>459</v>
       </c>
       <c r="C151" t="s">
-        <v>354</v>
+        <v>460</v>
       </c>
       <c r="D151" t="s">
-        <v>354</v>
+        <v>460</v>
       </c>
       <c r="E151" t="s">
         <v>160</v>
@@ -4279,13 +4153,13 @@
     </row>
     <row r="152" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B152" t="s">
-        <v>355</v>
+        <v>461</v>
       </c>
       <c r="C152" t="s">
-        <v>356</v>
+        <v>462</v>
       </c>
       <c r="D152" t="s">
-        <v>356</v>
+        <v>462</v>
       </c>
       <c r="E152" t="s">
         <v>160</v>
@@ -4293,13 +4167,13 @@
     </row>
     <row r="153" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B153" t="s">
-        <v>357</v>
+        <v>463</v>
       </c>
       <c r="C153" t="s">
-        <v>358</v>
+        <v>464</v>
       </c>
       <c r="D153" t="s">
-        <v>358</v>
+        <v>464</v>
       </c>
       <c r="E153" t="s">
         <v>160</v>
@@ -4307,13 +4181,13 @@
     </row>
     <row r="154" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B154" t="s">
-        <v>359</v>
+        <v>465</v>
       </c>
       <c r="C154" t="s">
-        <v>360</v>
+        <v>466</v>
       </c>
       <c r="D154" t="s">
-        <v>360</v>
+        <v>466</v>
       </c>
       <c r="E154" t="s">
         <v>160</v>
@@ -4321,13 +4195,13 @@
     </row>
     <row r="155" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B155" t="s">
-        <v>361</v>
+        <v>467</v>
       </c>
       <c r="C155" t="s">
-        <v>362</v>
+        <v>468</v>
       </c>
       <c r="D155" t="s">
-        <v>362</v>
+        <v>468</v>
       </c>
       <c r="E155" t="s">
         <v>160</v>
@@ -4335,13 +4209,13 @@
     </row>
     <row r="156" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B156" t="s">
-        <v>363</v>
+        <v>469</v>
       </c>
       <c r="C156" t="s">
-        <v>364</v>
+        <v>470</v>
       </c>
       <c r="D156" t="s">
-        <v>364</v>
+        <v>470</v>
       </c>
       <c r="E156" t="s">
         <v>160</v>
@@ -4349,13 +4223,13 @@
     </row>
     <row r="157" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B157" t="s">
-        <v>365</v>
+        <v>471</v>
       </c>
       <c r="C157" t="s">
-        <v>366</v>
+        <v>472</v>
       </c>
       <c r="D157" t="s">
-        <v>366</v>
+        <v>472</v>
       </c>
       <c r="E157" t="s">
         <v>160</v>
@@ -4363,13 +4237,13 @@
     </row>
     <row r="158" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B158" t="s">
-        <v>367</v>
+        <v>473</v>
       </c>
       <c r="C158" t="s">
-        <v>368</v>
+        <v>474</v>
       </c>
       <c r="D158" t="s">
-        <v>368</v>
+        <v>474</v>
       </c>
       <c r="E158" t="s">
         <v>160</v>
@@ -4377,13 +4251,13 @@
     </row>
     <row r="159" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B159" t="s">
-        <v>369</v>
+        <v>475</v>
       </c>
       <c r="C159" t="s">
-        <v>370</v>
+        <v>476</v>
       </c>
       <c r="D159" t="s">
-        <v>370</v>
+        <v>476</v>
       </c>
       <c r="E159" t="s">
         <v>160</v>
@@ -4391,13 +4265,13 @@
     </row>
     <row r="160" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B160" t="s">
-        <v>371</v>
+        <v>477</v>
       </c>
       <c r="C160" t="s">
-        <v>372</v>
+        <v>478</v>
       </c>
       <c r="D160" t="s">
-        <v>372</v>
+        <v>478</v>
       </c>
       <c r="E160" t="s">
         <v>160</v>
@@ -4405,13 +4279,13 @@
     </row>
     <row r="161" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B161" t="s">
-        <v>373</v>
+        <v>479</v>
       </c>
       <c r="C161" t="s">
-        <v>374</v>
+        <v>480</v>
       </c>
       <c r="D161" t="s">
-        <v>374</v>
+        <v>480</v>
       </c>
       <c r="E161" t="s">
         <v>160</v>
@@ -4419,13 +4293,13 @@
     </row>
     <row r="162" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B162" t="s">
-        <v>375</v>
+        <v>481</v>
       </c>
       <c r="C162" t="s">
-        <v>376</v>
+        <v>482</v>
       </c>
       <c r="D162" t="s">
-        <v>376</v>
+        <v>482</v>
       </c>
       <c r="E162" t="s">
         <v>160</v>
@@ -4433,13 +4307,13 @@
     </row>
     <row r="163" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B163" t="s">
-        <v>377</v>
+        <v>483</v>
       </c>
       <c r="C163" t="s">
-        <v>378</v>
+        <v>484</v>
       </c>
       <c r="D163" t="s">
-        <v>378</v>
+        <v>484</v>
       </c>
       <c r="E163" t="s">
         <v>160</v>
@@ -4447,13 +4321,13 @@
     </row>
     <row r="164" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B164" t="s">
-        <v>379</v>
+        <v>485</v>
       </c>
       <c r="C164" t="s">
-        <v>380</v>
+        <v>486</v>
       </c>
       <c r="D164" t="s">
-        <v>380</v>
+        <v>486</v>
       </c>
       <c r="E164" t="s">
         <v>160</v>
@@ -4461,13 +4335,13 @@
     </row>
     <row r="165" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B165" t="s">
-        <v>381</v>
+        <v>487</v>
       </c>
       <c r="C165" t="s">
-        <v>382</v>
+        <v>488</v>
       </c>
       <c r="D165" t="s">
-        <v>382</v>
+        <v>488</v>
       </c>
       <c r="E165" t="s">
         <v>160</v>
@@ -4475,13 +4349,13 @@
     </row>
     <row r="166" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B166" t="s">
-        <v>383</v>
+        <v>489</v>
       </c>
       <c r="C166" t="s">
-        <v>384</v>
+        <v>490</v>
       </c>
       <c r="D166" t="s">
-        <v>384</v>
+        <v>490</v>
       </c>
       <c r="E166" t="s">
         <v>160</v>
@@ -4489,13 +4363,13 @@
     </row>
     <row r="167" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B167" t="s">
-        <v>385</v>
+        <v>491</v>
       </c>
       <c r="C167" t="s">
-        <v>386</v>
+        <v>492</v>
       </c>
       <c r="D167" t="s">
-        <v>386</v>
+        <v>492</v>
       </c>
       <c r="E167" t="s">
         <v>160</v>
@@ -4657,13 +4531,13 @@
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B179" t="s">
-        <v>515</v>
+        <v>321</v>
       </c>
       <c r="C179" t="s">
-        <v>516</v>
+        <v>322</v>
       </c>
       <c r="D179" t="s">
-        <v>516</v>
+        <v>322</v>
       </c>
       <c r="E179" t="s">
         <v>160</v>
@@ -4671,13 +4545,13 @@
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B180" t="s">
-        <v>517</v>
+        <v>323</v>
       </c>
       <c r="C180" t="s">
-        <v>518</v>
+        <v>324</v>
       </c>
       <c r="D180" t="s">
-        <v>518</v>
+        <v>324</v>
       </c>
       <c r="E180" t="s">
         <v>160</v>
@@ -4685,13 +4559,13 @@
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B181" t="s">
-        <v>519</v>
+        <v>325</v>
       </c>
       <c r="C181" t="s">
-        <v>520</v>
+        <v>326</v>
       </c>
       <c r="D181" t="s">
-        <v>520</v>
+        <v>326</v>
       </c>
       <c r="E181" t="s">
         <v>160</v>
@@ -4699,13 +4573,13 @@
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B182" t="s">
-        <v>521</v>
+        <v>327</v>
       </c>
       <c r="C182" t="s">
-        <v>522</v>
+        <v>328</v>
       </c>
       <c r="D182" t="s">
-        <v>522</v>
+        <v>328</v>
       </c>
       <c r="E182" t="s">
         <v>160</v>
@@ -4713,13 +4587,13 @@
     </row>
     <row r="183" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B183" t="s">
-        <v>523</v>
+        <v>329</v>
       </c>
       <c r="C183" t="s">
-        <v>524</v>
+        <v>330</v>
       </c>
       <c r="D183" t="s">
-        <v>524</v>
+        <v>330</v>
       </c>
       <c r="E183" t="s">
         <v>160</v>
@@ -4727,13 +4601,13 @@
     </row>
     <row r="184" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B184" t="s">
-        <v>525</v>
+        <v>331</v>
       </c>
       <c r="C184" t="s">
-        <v>526</v>
+        <v>332</v>
       </c>
       <c r="D184" t="s">
-        <v>526</v>
+        <v>332</v>
       </c>
       <c r="E184" t="s">
         <v>160</v>
@@ -4741,13 +4615,13 @@
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B185" t="s">
-        <v>527</v>
+        <v>333</v>
       </c>
       <c r="C185" t="s">
-        <v>528</v>
+        <v>334</v>
       </c>
       <c r="D185" t="s">
-        <v>528</v>
+        <v>334</v>
       </c>
       <c r="E185" t="s">
         <v>160</v>
@@ -4755,13 +4629,13 @@
     </row>
     <row r="186" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B186" t="s">
-        <v>529</v>
+        <v>335</v>
       </c>
       <c r="C186" t="s">
-        <v>530</v>
+        <v>336</v>
       </c>
       <c r="D186" t="s">
-        <v>530</v>
+        <v>336</v>
       </c>
       <c r="E186" t="s">
         <v>160</v>
@@ -4769,13 +4643,13 @@
     </row>
     <row r="187" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B187" t="s">
-        <v>531</v>
+        <v>337</v>
       </c>
       <c r="C187" t="s">
-        <v>532</v>
+        <v>338</v>
       </c>
       <c r="D187" t="s">
-        <v>532</v>
+        <v>338</v>
       </c>
       <c r="E187" t="s">
         <v>160</v>
@@ -4783,309 +4657,15 @@
     </row>
     <row r="188" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B188" t="s">
-        <v>533</v>
+        <v>339</v>
       </c>
       <c r="C188" t="s">
-        <v>534</v>
+        <v>340</v>
       </c>
       <c r="D188" t="s">
-        <v>534</v>
+        <v>340</v>
       </c>
       <c r="E188" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="189" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B189" t="s">
-        <v>535</v>
-      </c>
-      <c r="C189" t="s">
-        <v>536</v>
-      </c>
-      <c r="D189" t="s">
-        <v>536</v>
-      </c>
-      <c r="E189" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="190" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B190" t="s">
-        <v>537</v>
-      </c>
-      <c r="C190" t="s">
-        <v>538</v>
-      </c>
-      <c r="D190" t="s">
-        <v>538</v>
-      </c>
-      <c r="E190" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="191" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B191" t="s">
-        <v>539</v>
-      </c>
-      <c r="C191" t="s">
-        <v>540</v>
-      </c>
-      <c r="D191" t="s">
-        <v>540</v>
-      </c>
-      <c r="E191" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="192" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B192" t="s">
-        <v>541</v>
-      </c>
-      <c r="C192" t="s">
-        <v>542</v>
-      </c>
-      <c r="D192" t="s">
-        <v>542</v>
-      </c>
-      <c r="E192" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="193" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B193" t="s">
-        <v>543</v>
-      </c>
-      <c r="C193" t="s">
-        <v>544</v>
-      </c>
-      <c r="D193" t="s">
-        <v>544</v>
-      </c>
-      <c r="E193" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="194" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B194" t="s">
-        <v>545</v>
-      </c>
-      <c r="C194" t="s">
-        <v>546</v>
-      </c>
-      <c r="D194" t="s">
-        <v>546</v>
-      </c>
-      <c r="E194" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="195" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B195" t="s">
-        <v>547</v>
-      </c>
-      <c r="C195" t="s">
-        <v>548</v>
-      </c>
-      <c r="D195" t="s">
-        <v>548</v>
-      </c>
-      <c r="E195" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="196" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B196" t="s">
-        <v>549</v>
-      </c>
-      <c r="C196" t="s">
-        <v>550</v>
-      </c>
-      <c r="D196" t="s">
-        <v>550</v>
-      </c>
-      <c r="E196" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="197" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B197" t="s">
-        <v>551</v>
-      </c>
-      <c r="C197" t="s">
-        <v>552</v>
-      </c>
-      <c r="D197" t="s">
-        <v>552</v>
-      </c>
-      <c r="E197" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="198" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B198" t="s">
-        <v>553</v>
-      </c>
-      <c r="C198" t="s">
-        <v>554</v>
-      </c>
-      <c r="D198" t="s">
-        <v>554</v>
-      </c>
-      <c r="E198" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="199" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B199" t="s">
-        <v>555</v>
-      </c>
-      <c r="C199" t="s">
-        <v>556</v>
-      </c>
-      <c r="D199" t="s">
-        <v>556</v>
-      </c>
-      <c r="E199" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="200" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B200" t="s">
-        <v>387</v>
-      </c>
-      <c r="C200" t="s">
-        <v>388</v>
-      </c>
-      <c r="D200" t="s">
-        <v>388</v>
-      </c>
-      <c r="E200" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="201" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B201" t="s">
-        <v>389</v>
-      </c>
-      <c r="C201" t="s">
-        <v>390</v>
-      </c>
-      <c r="D201" t="s">
-        <v>390</v>
-      </c>
-      <c r="E201" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="202" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B202" t="s">
-        <v>391</v>
-      </c>
-      <c r="C202" t="s">
-        <v>392</v>
-      </c>
-      <c r="D202" t="s">
-        <v>392</v>
-      </c>
-      <c r="E202" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="203" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B203" t="s">
-        <v>393</v>
-      </c>
-      <c r="C203" t="s">
-        <v>394</v>
-      </c>
-      <c r="D203" t="s">
-        <v>394</v>
-      </c>
-      <c r="E203" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="204" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B204" t="s">
-        <v>395</v>
-      </c>
-      <c r="C204" t="s">
-        <v>396</v>
-      </c>
-      <c r="D204" t="s">
-        <v>396</v>
-      </c>
-      <c r="E204" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="205" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B205" t="s">
-        <v>397</v>
-      </c>
-      <c r="C205" t="s">
-        <v>398</v>
-      </c>
-      <c r="D205" t="s">
-        <v>398</v>
-      </c>
-      <c r="E205" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="206" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B206" t="s">
-        <v>399</v>
-      </c>
-      <c r="C206" t="s">
-        <v>400</v>
-      </c>
-      <c r="D206" t="s">
-        <v>400</v>
-      </c>
-      <c r="E206" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="207" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B207" t="s">
-        <v>401</v>
-      </c>
-      <c r="C207" t="s">
-        <v>402</v>
-      </c>
-      <c r="D207" t="s">
-        <v>402</v>
-      </c>
-      <c r="E207" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="208" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B208" t="s">
-        <v>403</v>
-      </c>
-      <c r="C208" t="s">
-        <v>404</v>
-      </c>
-      <c r="D208" t="s">
-        <v>404</v>
-      </c>
-      <c r="E208" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="209" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B209" t="s">
-        <v>405</v>
-      </c>
-      <c r="C209" t="s">
-        <v>406</v>
-      </c>
-      <c r="D209" t="s">
-        <v>406</v>
-      </c>
-      <c r="E209" t="s">
         <v>160</v>
       </c>
     </row>

</xml_diff>